<commit_message>
docs: update smart feature dry run reports
</commit_message>
<xml_diff>
--- a/wings_control/docs/rebuild-260715/AI Infra工作台_0 Day测试结果_白名单差异场景及优化参数.xlsx
+++ b/wings_control/docs/rebuild-260715/AI Infra工作台_0 Day测试结果_白名单差异场景及优化参数.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\wings-k8s-260703\wings_control\docs\rebuild-260715\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531BF90D-2A97-414B-A8DD-94916A332FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E239C9ED-C812-42A7-89C3-D741CD9ABF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="21806" windowHeight="13886" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="21806" windowHeight="13886" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="白名单差异场景" sheetId="1" r:id="rId1"/>
@@ -19,11 +19,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">白名单差异场景!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>官方开源模型名称（源D列）</t>
   </si>
@@ -35,9 +36,6 @@
   </si>
   <si>
     <t>优化拉起参数（源Q列）</t>
-  </si>
-  <si>
-    <t>Qwen3.6-27B</t>
   </si>
   <si>
     <t>Native卸载,
@@ -816,157 +814,157 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="C11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>